<commit_message>
fix(fixtures): backfill pattern.version into all draft patterns
All 22 pattern-from-draft.xlsx (and their CSV twins) were missing the
config: | pattern.version | 1 row. The drafter stamps it for new runs
but existing fixtures predated or bypassed the stamp.

Added by inserting row 1 in each file; extraction output is unchanged.

Also synced bundled examples:
- 03_expense_report/pattern.xlsx -> 05_expense_report manual pattern
- grepxcel/examples/ (03, 04) re-synced to find_pattern_xlsx() output

1561 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/01_simple_invoice/01_simple_invoice_pattern-from-draft.xlsx
+++ b/tests/fixtures/01_simple_invoice/01_simple_invoice_pattern-from-draft.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -447,22 +447,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>read.direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="n"/>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>pattern.version</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -472,37 +471,33 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
+          <t>read.direction</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>config:</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
           <t>currency.sign</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>inv.number</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>[A-Z]{2}[0-9]{6}</t>
-        </is>
-      </c>
+      <c r="D3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -512,17 +507,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>inv.date</t>
+          <t>inv.number</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>.*</t>
+          <t>[A-Z]{2}[0-9]{6}</t>
         </is>
       </c>
     </row>
@@ -534,7 +529,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>inv.due_date</t>
+          <t>inv.date</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -556,17 +551,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>client.name</t>
+          <t>inv.due_date</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>.+</t>
+          <t>.*</t>
         </is>
       </c>
     </row>
@@ -578,7 +573,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>client.email</t>
+          <t>client.name</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -588,7 +583,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>.+@.+</t>
+          <t>.+</t>
         </is>
       </c>
     </row>
@@ -600,17 +595,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>amount.net</t>
+          <t>client.email</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>.*</t>
+          <t>.+@.+</t>
         </is>
       </c>
     </row>
@@ -622,7 +617,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>amount.vat</t>
+          <t>amount.net</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -644,43 +639,51 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>amount.vat</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>.*</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
           <t>amount.gross</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>START:</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -690,7 +693,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>inv.number</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C13" s="4" t="n"/>
@@ -704,7 +707,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>inv.number</t>
         </is>
       </c>
       <c r="C14" s="4" t="n"/>
@@ -718,7 +721,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>inv.date</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C15" s="4" t="n"/>
@@ -732,7 +735,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>inv.date</t>
         </is>
       </c>
       <c r="C16" s="4" t="n"/>
@@ -746,7 +749,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>inv.due_date</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C17" s="4" t="n"/>
@@ -760,7 +763,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>inv.due_date</t>
         </is>
       </c>
       <c r="C18" s="4" t="n"/>
@@ -774,7 +777,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>client.name</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C19" s="4" t="n"/>
@@ -788,7 +791,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>client.name</t>
         </is>
       </c>
       <c r="C20" s="4" t="n"/>
@@ -802,7 +805,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>client.email</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C21" s="4" t="n"/>
@@ -816,7 +819,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>client.email</t>
         </is>
       </c>
       <c r="C22" s="4" t="n"/>
@@ -830,7 +833,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>amount.net</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C23" s="4" t="n"/>
@@ -844,7 +847,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>amount.net</t>
         </is>
       </c>
       <c r="C24" s="4" t="n"/>
@@ -858,7 +861,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>amount.vat</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C25" s="4" t="n"/>
@@ -872,7 +875,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>IGNORE</t>
+          <t>amount.vat</t>
         </is>
       </c>
       <c r="C26" s="4" t="n"/>
@@ -886,21 +889,35 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>amount.gross</t>
+          <t>IGNORE</t>
         </is>
       </c>
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>amount.gross</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>END:</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(generate_fixtures): colorize draft patterns on generation; sync examples
generate_fixtures.py now calls colorize_pattern_file() after saving each
pattern-from-draft.xlsx, matching the behaviour of the drafter.py CLI path.
Previously the 14 programmatically-generated draft patterns were plain
(no fill colours), while claude/local patterns produced via 'grepxcel draft'
were coloured. Now all draft patterns are consistently coloured.

Also re-syncs grepxcel/examples/*/data.xlsx after the second regeneration
run (ZIP timestamps changed).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/01_simple_invoice/01_simple_invoice_pattern-from-draft.xlsx
+++ b/tests/fixtures/01_simple_invoice/01_simple_invoice_pattern-from-draft.xlsx
@@ -26,12 +26,32 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE8D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0FFD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0E0FF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +66,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,422 +439,468 @@
   </sheetPr>
   <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>read.direction</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>LR</t>
         </is>
       </c>
+      <c r="D1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>config:</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>currency.sign</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
+      <c r="D2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>inv.number</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>[A-Z]{2}[0-9]{6}</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>inv.date</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>inv.due_date</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>client.name</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>.+</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>client.email</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>.+@.+</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>amount.net</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>amount.vat</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>var:</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>amount.gross</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>.*</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>START:</t>
         </is>
       </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>inv.number</t>
         </is>
       </c>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>inv.date</t>
         </is>
       </c>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>inv.due_date</t>
         </is>
       </c>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>client.name</t>
         </is>
       </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>client.email</t>
         </is>
       </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>amount.net</t>
         </is>
       </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>amount.vat</t>
         </is>
       </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>IGNORE</t>
         </is>
       </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>cell:1</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>cell:1</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>amount.gross</t>
         </is>
       </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>END:</t>
         </is>
       </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>